<commit_message>
feat(schema): wire group context through workbook builders
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report.xlsx
+++ b/packages/typed-xlsx/examples/financial-report.xlsx
@@ -40,127 +40,127 @@
     <t>Average Profit Margin</t>
   </si>
   <si>
-    <t>2023-03</t>
+    <t>2023-09</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>35.3%</t>
+  </si>
+  <si>
+    <t>71.74%</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>75.69%</t>
+  </si>
+  <si>
+    <t>2023-11</t>
+  </si>
+  <si>
+    <t>68.99%</t>
   </si>
   <si>
     <t>R&amp;D</t>
   </si>
   <si>
-    <t>91.27%</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>-24.68%</t>
-  </si>
-  <si>
-    <t>79.28%</t>
-  </si>
-  <si>
-    <t>2023-12</t>
-  </si>
-  <si>
-    <t>78.54%</t>
-  </si>
-  <si>
-    <t>14.6%</t>
-  </si>
-  <si>
-    <t>-40.94%</t>
+    <t>89.65%</t>
+  </si>
+  <si>
+    <t>68.71%</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>-47.54%</t>
+  </si>
+  <si>
+    <t>12.47%</t>
+  </si>
+  <si>
+    <t>-81.36%</t>
+  </si>
+  <si>
+    <t>2023-06</t>
+  </si>
+  <si>
+    <t>10.05%</t>
+  </si>
+  <si>
+    <t>43.73%</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>11.46%</t>
+  </si>
+  <si>
+    <t>2023-10</t>
+  </si>
+  <si>
+    <t>46.02%</t>
+  </si>
+  <si>
+    <t>83.05%</t>
+  </si>
+  <si>
+    <t>77.52%</t>
+  </si>
+  <si>
+    <t>73.46%</t>
+  </si>
+  <si>
+    <t>80.59%</t>
+  </si>
+  <si>
+    <t>13.49%</t>
+  </si>
+  <si>
+    <t>87.92%</t>
+  </si>
+  <si>
+    <t>51.24%</t>
+  </si>
+  <si>
+    <t>56.27%</t>
+  </si>
+  <si>
+    <t>-23.92%</t>
+  </si>
+  <si>
+    <t>75.62%</t>
+  </si>
+  <si>
+    <t>73.9%</t>
   </si>
   <si>
     <t>2023-01</t>
   </si>
   <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>-344.04%</t>
-  </si>
-  <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>44.6%</t>
-  </si>
-  <si>
-    <t>55.78%</t>
-  </si>
-  <si>
-    <t>2023-09</t>
-  </si>
-  <si>
-    <t>-15.48%</t>
-  </si>
-  <si>
-    <t>59.77%</t>
-  </si>
-  <si>
-    <t>60.15%</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>67.36%</t>
-  </si>
-  <si>
-    <t>81.24%</t>
-  </si>
-  <si>
-    <t>73.18%</t>
-  </si>
-  <si>
-    <t>65.57%</t>
-  </si>
-  <si>
-    <t>48.27%</t>
-  </si>
-  <si>
-    <t>7.78%</t>
-  </si>
-  <si>
-    <t>2023-07</t>
-  </si>
-  <si>
-    <t>-82.94%</t>
-  </si>
-  <si>
-    <t>5.66%</t>
-  </si>
-  <si>
-    <t>71.33%</t>
-  </si>
-  <si>
-    <t>-13.35%</t>
-  </si>
-  <si>
-    <t>64.4%</t>
-  </si>
-  <si>
-    <t>72.75%</t>
-  </si>
-  <si>
-    <t>2023-04</t>
-  </si>
-  <si>
-    <t>-78.65%</t>
-  </si>
-  <si>
-    <t>51.7%</t>
-  </si>
-  <si>
-    <t>78.77%</t>
-  </si>
-  <si>
-    <t>-45.03%</t>
-  </si>
-  <si>
-    <t>81.95%</t>
-  </si>
-  <si>
-    <t>63.36%</t>
+    <t>93.9%</t>
+  </si>
+  <si>
+    <t>71.07%</t>
+  </si>
+  <si>
+    <t>10.19%</t>
+  </si>
+  <si>
+    <t>2023-08</t>
+  </si>
+  <si>
+    <t>20.92%</t>
+  </si>
+  <si>
+    <t>78.91%</t>
+  </si>
+  <si>
+    <t>34.51%</t>
   </si>
 </sst>
 </file>
@@ -350,46 +350,46 @@
         <v>11</v>
       </c>
       <c r="C2" s="3">
-        <v>97757</v>
+        <v>45932</v>
       </c>
       <c r="D2" s="3">
-        <v>8533</v>
+        <v>29720</v>
       </c>
       <c r="E2" s="4">
-        <v>89224</v>
+        <v>16212</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>12</v>
       </c>
       <c r="G2" s="3">
-        <v>214472</v>
+        <v>176453</v>
       </c>
       <c r="H2" s="3">
-        <v>60476</v>
+        <v>65146</v>
       </c>
       <c r="I2" s="4">
-        <v>153996</v>
+        <v>111307</v>
       </c>
       <c r="J2" s="6">
-        <v>48.623333333333335</v>
+        <v>60.91</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2"/>
       <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3">
+        <v>93574</v>
+      </c>
+      <c r="D3" s="3">
+        <v>26444</v>
+      </c>
+      <c r="E3" s="4">
+        <v>67130</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" s="3">
-        <v>26705</v>
-      </c>
-      <c r="D3" s="3">
-        <v>33297</v>
-      </c>
-      <c r="E3" s="7">
-        <v>-6592</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -399,16 +399,16 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3">
-        <v>90010</v>
+        <v>36947</v>
       </c>
       <c r="D4" s="3">
-        <v>18646</v>
+        <v>8982</v>
       </c>
       <c r="E4" s="4">
-        <v>71364</v>
+        <v>27965</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>15</v>
@@ -423,49 +423,49 @@
         <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" s="3">
-        <v>80355</v>
+        <v>44669</v>
       </c>
       <c r="D5" s="3">
-        <v>17248</v>
+        <v>13852</v>
       </c>
       <c r="E5" s="4">
-        <v>63107</v>
+        <v>30817</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="3">
-        <v>140230</v>
+        <v>162292</v>
       </c>
       <c r="H5" s="3">
-        <v>83927</v>
+        <v>33741</v>
       </c>
       <c r="I5" s="4">
-        <v>56303</v>
+        <v>128551</v>
       </c>
       <c r="J5" s="6">
-        <v>17.400000000000002</v>
+        <v>75.78333333333332</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C6" s="3">
-        <v>31880</v>
+        <v>80761</v>
       </c>
       <c r="D6" s="3">
-        <v>27224</v>
+        <v>8356</v>
       </c>
       <c r="E6" s="4">
-        <v>4656</v>
+        <v>72405</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
@@ -475,19 +475,19 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C7" s="3">
-        <v>27995</v>
+        <v>36862</v>
       </c>
       <c r="D7" s="3">
-        <v>39455</v>
-      </c>
-      <c r="E7" s="7">
-        <v>-11460</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>19</v>
+        <v>11533</v>
+      </c>
+      <c r="E7" s="4">
+        <v>25329</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
@@ -496,128 +496,128 @@
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="3">
-        <v>10898</v>
+        <v>16176</v>
       </c>
       <c r="D8" s="3">
-        <v>48391</v>
+        <v>23866</v>
       </c>
       <c r="E8" s="7">
-        <v>-37493</v>
+        <v>-7690</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>22</v>
       </c>
       <c r="G8" s="3">
-        <v>114191</v>
+        <v>86297</v>
       </c>
       <c r="H8" s="3">
-        <v>101276</v>
-      </c>
-      <c r="I8" s="4">
-        <v>12915</v>
+        <v>107163</v>
+      </c>
+      <c r="I8" s="7">
+        <v>-20866</v>
       </c>
       <c r="J8" s="9">
-        <v>-81.22</v>
+        <v>-38.81</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3">
+        <v>46759</v>
+      </c>
+      <c r="D9" s="3">
+        <v>40927</v>
+      </c>
+      <c r="E9" s="4">
+        <v>5832</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="C9" s="3">
-        <v>64453</v>
-      </c>
-      <c r="D9" s="3">
-        <v>35709</v>
-      </c>
-      <c r="E9" s="4">
-        <v>28744</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
-      <c r="I9" s="4"/>
+      <c r="I9" s="7"/>
       <c r="J9" s="9"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C10" s="3">
-        <v>38840</v>
+        <v>23362</v>
       </c>
       <c r="D10" s="3">
-        <v>17176</v>
-      </c>
-      <c r="E10" s="4">
-        <v>21664</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>25</v>
+        <v>42370</v>
+      </c>
+      <c r="E10" s="7">
+        <v>-19008</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
-      <c r="I10" s="4"/>
+      <c r="I10" s="7"/>
       <c r="J10" s="9"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="3">
+        <v>28413</v>
+      </c>
+      <c r="D11" s="3">
+        <v>25558</v>
+      </c>
+      <c r="E11" s="4">
+        <v>2855</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="3">
-        <v>12433</v>
-      </c>
-      <c r="D11" s="3">
-        <v>14358</v>
-      </c>
-      <c r="E11" s="7">
-        <v>-1925</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>27</v>
-      </c>
       <c r="G11" s="3">
-        <v>210369</v>
+        <v>130652</v>
       </c>
       <c r="H11" s="3">
-        <v>93615</v>
+        <v>99731</v>
       </c>
       <c r="I11" s="4">
-        <v>116754</v>
+        <v>30921</v>
       </c>
       <c r="J11" s="6">
-        <v>34.81333333333333</v>
+        <v>21.74666666666667</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C12" s="3">
-        <v>99940</v>
+        <v>50658</v>
       </c>
       <c r="D12" s="3">
-        <v>40205</v>
+        <v>28503</v>
       </c>
       <c r="E12" s="4">
-        <v>59735</v>
+        <v>22155</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
@@ -627,16 +627,16 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C13" s="3">
-        <v>97996</v>
+        <v>51581</v>
       </c>
       <c r="D13" s="3">
-        <v>39052</v>
+        <v>45670</v>
       </c>
       <c r="E13" s="4">
-        <v>58944</v>
+        <v>5911</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>29</v>
@@ -648,49 +648,49 @@
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C14" s="3">
-        <v>53082</v>
+        <v>83955</v>
       </c>
       <c r="D14" s="3">
-        <v>17328</v>
+        <v>45316</v>
       </c>
       <c r="E14" s="4">
-        <v>35754</v>
+        <v>38639</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>31</v>
       </c>
       <c r="G14" s="3">
-        <v>204111</v>
+        <v>219794</v>
       </c>
       <c r="H14" s="3">
-        <v>52802</v>
+        <v>71549</v>
       </c>
       <c r="I14" s="4">
-        <v>151309</v>
+        <v>148245</v>
       </c>
       <c r="J14" s="6">
-        <v>73.92666666666666</v>
+        <v>68.86333333333333</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C15" s="3">
-        <v>62389</v>
+        <v>77813</v>
       </c>
       <c r="D15" s="3">
-        <v>11704</v>
+        <v>13191</v>
       </c>
       <c r="E15" s="4">
-        <v>50685</v>
+        <v>64622</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>32</v>
@@ -703,16 +703,16 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C16" s="3">
-        <v>88640</v>
+        <v>58026</v>
       </c>
       <c r="D16" s="3">
-        <v>23770</v>
+        <v>13042</v>
       </c>
       <c r="E16" s="4">
-        <v>64870</v>
+        <v>44984</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>33</v>
@@ -724,49 +724,49 @@
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C17" s="3">
-        <v>57215</v>
+        <v>69394</v>
       </c>
       <c r="D17" s="3">
-        <v>19699</v>
+        <v>18414</v>
       </c>
       <c r="E17" s="4">
-        <v>37516</v>
+        <v>50980</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>34</v>
       </c>
       <c r="G17" s="3">
-        <v>178417</v>
+        <v>188442</v>
       </c>
       <c r="H17" s="3">
-        <v>104058</v>
+        <v>54363</v>
       </c>
       <c r="I17" s="4">
-        <v>74359</v>
+        <v>134079</v>
       </c>
       <c r="J17" s="6">
-        <v>40.54</v>
+        <v>55.84666666666667</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C18" s="3">
-        <v>67698</v>
+        <v>99916</v>
       </c>
       <c r="D18" s="3">
-        <v>35020</v>
+        <v>19397</v>
       </c>
       <c r="E18" s="4">
-        <v>32678</v>
+        <v>80519</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>35</v>
@@ -779,16 +779,16 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C19" s="3">
-        <v>53504</v>
+        <v>19132</v>
       </c>
       <c r="D19" s="3">
-        <v>49339</v>
+        <v>16552</v>
       </c>
       <c r="E19" s="4">
-        <v>4165</v>
+        <v>2580</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>36</v>
@@ -800,128 +800,128 @@
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C20" s="3">
-        <v>24748</v>
+        <v>74376</v>
       </c>
       <c r="D20" s="3">
-        <v>45275</v>
-      </c>
-      <c r="E20" s="7">
-        <v>-20527</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>38</v>
+        <v>8981</v>
+      </c>
+      <c r="E20" s="4">
+        <v>65395</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="G20" s="3">
-        <v>138205</v>
+        <v>206932</v>
       </c>
       <c r="H20" s="3">
-        <v>106621</v>
+        <v>71835</v>
       </c>
       <c r="I20" s="4">
-        <v>31584</v>
-      </c>
-      <c r="J20" s="9">
-        <v>-1.9833333333333343</v>
+        <v>135097</v>
+      </c>
+      <c r="J20" s="6">
+        <v>65.14333333333333</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C21" s="3">
-        <v>43888</v>
+        <v>97093</v>
       </c>
       <c r="D21" s="3">
-        <v>41403</v>
+        <v>47345</v>
       </c>
       <c r="E21" s="4">
-        <v>2485</v>
+        <v>49748</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="9"/>
+      <c r="J21" s="6"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C22" s="3">
-        <v>69569</v>
+        <v>35463</v>
       </c>
       <c r="D22" s="3">
-        <v>19943</v>
+        <v>15509</v>
       </c>
       <c r="E22" s="4">
-        <v>49626</v>
+        <v>19954</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
       <c r="I22" s="4"/>
-      <c r="J22" s="9"/>
+      <c r="J22" s="6"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C23" s="3">
-        <v>39117</v>
+        <v>24628</v>
       </c>
       <c r="D23" s="3">
-        <v>44340</v>
+        <v>30519</v>
       </c>
       <c r="E23" s="7">
-        <v>-5223</v>
+        <v>-5891</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G23" s="3">
-        <v>172263</v>
+        <v>163123</v>
       </c>
       <c r="H23" s="3">
-        <v>87506</v>
+        <v>65814</v>
       </c>
       <c r="I23" s="4">
-        <v>84757</v>
+        <v>97309</v>
       </c>
       <c r="J23" s="6">
-        <v>41.26666666666667</v>
+        <v>41.86666666666667</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="C24" s="3">
-        <v>82486</v>
+        <v>49590</v>
       </c>
       <c r="D24" s="3">
-        <v>29363</v>
+        <v>12091</v>
       </c>
       <c r="E24" s="4">
-        <v>53123</v>
+        <v>37499</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
@@ -934,16 +934,16 @@
         <v>21</v>
       </c>
       <c r="C25" s="3">
-        <v>50660</v>
+        <v>88905</v>
       </c>
       <c r="D25" s="3">
-        <v>13803</v>
+        <v>23204</v>
       </c>
       <c r="E25" s="4">
-        <v>36857</v>
+        <v>65701</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
@@ -952,52 +952,52 @@
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="3">
+        <v>84708</v>
+      </c>
+      <c r="D26" s="3">
+        <v>5166</v>
+      </c>
+      <c r="E26" s="4">
+        <v>79542</v>
+      </c>
+      <c r="F26" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="3">
-        <v>17966</v>
-      </c>
-      <c r="D26" s="3">
-        <v>32096</v>
-      </c>
-      <c r="E26" s="7">
-        <v>-14130</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>45</v>
-      </c>
       <c r="G26" s="3">
-        <v>172235</v>
+        <v>181037</v>
       </c>
       <c r="H26" s="3">
-        <v>80022</v>
+        <v>43950</v>
       </c>
       <c r="I26" s="4">
-        <v>92213</v>
+        <v>137087</v>
       </c>
       <c r="J26" s="6">
-        <v>17.27333333333333</v>
+        <v>58.38666666666666</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C27" s="3">
-        <v>56074</v>
+        <v>78395</v>
       </c>
       <c r="D27" s="3">
-        <v>27084</v>
+        <v>22678</v>
       </c>
       <c r="E27" s="4">
-        <v>28990</v>
+        <v>55717</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
@@ -1007,19 +1007,19 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C28" s="3">
-        <v>98195</v>
+        <v>17934</v>
       </c>
       <c r="D28" s="3">
-        <v>20842</v>
+        <v>16106</v>
       </c>
       <c r="E28" s="4">
-        <v>77353</v>
+        <v>1828</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
@@ -1028,49 +1028,49 @@
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C29" s="3">
-        <v>22197</v>
+        <v>62750</v>
       </c>
       <c r="D29" s="3">
-        <v>32192</v>
-      </c>
-      <c r="E29" s="7">
-        <v>-9995</v>
-      </c>
-      <c r="F29" s="8" t="s">
+        <v>49625</v>
+      </c>
+      <c r="E29" s="4">
+        <v>13125</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>48</v>
       </c>
       <c r="G29" s="3">
-        <v>144064</v>
+        <v>170563</v>
       </c>
       <c r="H29" s="3">
-        <v>64883</v>
+        <v>77306</v>
       </c>
       <c r="I29" s="4">
-        <v>79181</v>
+        <v>93257</v>
       </c>
       <c r="J29" s="6">
-        <v>33.42666666666667</v>
+        <v>44.78</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="C30" s="3">
-        <v>64335</v>
+        <v>96688</v>
       </c>
       <c r="D30" s="3">
-        <v>11614</v>
+        <v>20395</v>
       </c>
       <c r="E30" s="4">
-        <v>52721</v>
+        <v>76293</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>49</v>
@@ -1083,16 +1083,16 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C31" s="3">
-        <v>57532</v>
+        <v>11125</v>
       </c>
       <c r="D31" s="3">
-        <v>21077</v>
+        <v>7286</v>
       </c>
       <c r="E31" s="4">
-        <v>36455</v>
+        <v>3839</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>50</v>
@@ -1104,16 +1104,16 @@
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1688557</v>
+        <v>1685585</v>
       </c>
       <c r="H32" s="10">
-        <v>835186</v>
+        <v>690598</v>
       </c>
       <c r="I32" s="11">
-        <v>853371</v>
+        <v>994987</v>
       </c>
       <c r="J32" s="12">
-        <v>22.406666666666673</v>
+        <v>45.45166666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(examples): regenerate workbook artifacts
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report.xlsx
+++ b/packages/typed-xlsx/examples/financial-report.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Month</t>
   </si>
@@ -40,127 +40,130 @@
     <t>Average Profit Margin</t>
   </si>
   <si>
-    <t>2023-01</t>
+    <t>2023-11</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>9.86%</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>52.77%</t>
+  </si>
+  <si>
+    <t>-98.55%</t>
+  </si>
+  <si>
+    <t>2023-12</t>
+  </si>
+  <si>
+    <t>41.09%</t>
+  </si>
+  <si>
+    <t>R&amp;D</t>
+  </si>
+  <si>
+    <t>-53.75%</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>58.85%</t>
+  </si>
+  <si>
+    <t>2023-05</t>
+  </si>
+  <si>
+    <t>89.68%</t>
   </si>
   <si>
     <t>Sales</t>
   </si>
   <si>
-    <t>72.14%</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>66.28%</t>
-  </si>
-  <si>
-    <t>R&amp;D</t>
-  </si>
-  <si>
-    <t>15.55%</t>
+    <t>17.94%</t>
+  </si>
+  <si>
+    <t>63.39%</t>
+  </si>
+  <si>
+    <t>2023-08</t>
+  </si>
+  <si>
+    <t>-8.3%</t>
+  </si>
+  <si>
+    <t>44.61%</t>
+  </si>
+  <si>
+    <t>39.29%</t>
+  </si>
+  <si>
+    <t>42.39%</t>
+  </si>
+  <si>
+    <t>47.31%</t>
+  </si>
+  <si>
+    <t>59.77%</t>
+  </si>
+  <si>
+    <t>2023-10</t>
+  </si>
+  <si>
+    <t>31.86%</t>
+  </si>
+  <si>
+    <t>-237.28%</t>
+  </si>
+  <si>
+    <t>74.97%</t>
+  </si>
+  <si>
+    <t>2023-04</t>
+  </si>
+  <si>
+    <t>2.73%</t>
+  </si>
+  <si>
+    <t>-96.16%</t>
+  </si>
+  <si>
+    <t>45.4%</t>
+  </si>
+  <si>
+    <t>81.86%</t>
+  </si>
+  <si>
+    <t>47.81%</t>
+  </si>
+  <si>
+    <t>-30.43%</t>
   </si>
   <si>
     <t>2023-09</t>
   </si>
   <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>12.4%</t>
-  </si>
-  <si>
-    <t>84.26%</t>
-  </si>
-  <si>
-    <t>4.02%</t>
-  </si>
-  <si>
-    <t>49.98%</t>
-  </si>
-  <si>
-    <t>-24.58%</t>
-  </si>
-  <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>41.48%</t>
-  </si>
-  <si>
-    <t>57.18%</t>
-  </si>
-  <si>
-    <t>-128.81%</t>
-  </si>
-  <si>
-    <t>-51.13%</t>
-  </si>
-  <si>
-    <t>2023-07</t>
-  </si>
-  <si>
-    <t>83.99%</t>
-  </si>
-  <si>
-    <t>58.69%</t>
-  </si>
-  <si>
-    <t>46.82%</t>
-  </si>
-  <si>
-    <t>2023-04</t>
-  </si>
-  <si>
-    <t>-205.92%</t>
-  </si>
-  <si>
-    <t>65.31%</t>
-  </si>
-  <si>
-    <t>70.89%</t>
-  </si>
-  <si>
-    <t>2023-06</t>
-  </si>
-  <si>
-    <t>80.83%</t>
-  </si>
-  <si>
-    <t>45.12%</t>
-  </si>
-  <si>
-    <t>36.75%</t>
-  </si>
-  <si>
-    <t>44.34%</t>
-  </si>
-  <si>
-    <t>57.29%</t>
-  </si>
-  <si>
-    <t>91.91%</t>
-  </si>
-  <si>
-    <t>2023-03</t>
-  </si>
-  <si>
-    <t>86.25%</t>
-  </si>
-  <si>
-    <t>91.76%</t>
-  </si>
-  <si>
-    <t>78.01%</t>
-  </si>
-  <si>
-    <t>-104.98%</t>
-  </si>
-  <si>
-    <t>91.29%</t>
-  </si>
-  <si>
-    <t>1.61%</t>
+    <t>-138.16%</t>
+  </si>
+  <si>
+    <t>84.4%</t>
+  </si>
+  <si>
+    <t>82.12%</t>
+  </si>
+  <si>
+    <t>53.5%</t>
+  </si>
+  <si>
+    <t>-31.91%</t>
+  </si>
+  <si>
+    <t>37.13%</t>
   </si>
 </sst>
 </file>
@@ -269,7 +272,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -278,7 +281,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -354,28 +357,28 @@
         <v>11</v>
       </c>
       <c r="C2" s="3">
-        <v>49012</v>
+        <v>37960</v>
       </c>
       <c r="D2" s="3">
-        <v>13654</v>
+        <v>34219</v>
       </c>
       <c r="E2" s="4">
-        <v>35358</v>
+        <v>3741</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>12</v>
       </c>
       <c r="G2" s="3">
-        <v>101485</v>
+        <v>98357</v>
       </c>
       <c r="H2" s="3">
-        <v>38904</v>
+        <v>82432</v>
       </c>
       <c r="I2" s="4">
-        <v>62581</v>
+        <v>15925</v>
       </c>
       <c r="J2" s="6">
-        <v>51.323333333333345</v>
+        <v>-11.973333333333331</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -384,13 +387,13 @@
         <v>13</v>
       </c>
       <c r="C3" s="3">
-        <v>37579</v>
+        <v>47388</v>
       </c>
       <c r="D3" s="3">
-        <v>12672</v>
+        <v>22383</v>
       </c>
       <c r="E3" s="4">
-        <v>24907</v>
+        <v>25005</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>14</v>
@@ -403,19 +406,19 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3">
+        <v>13009</v>
+      </c>
+      <c r="D4" s="3">
+        <v>25830</v>
+      </c>
+      <c r="E4" s="7">
+        <v>-12821</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>15</v>
-      </c>
-      <c r="C4" s="3">
-        <v>14894</v>
-      </c>
-      <c r="D4" s="3">
-        <v>12578</v>
-      </c>
-      <c r="E4" s="4">
-        <v>2316</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>16</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -424,71 +427,71 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3">
+        <v>75872</v>
+      </c>
+      <c r="D5" s="3">
+        <v>44694</v>
+      </c>
+      <c r="E5" s="4">
+        <v>31178</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="3">
-        <v>42991</v>
-      </c>
-      <c r="D5" s="3">
-        <v>37660</v>
-      </c>
-      <c r="E5" s="4">
-        <v>5331</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>19</v>
-      </c>
       <c r="G5" s="3">
-        <v>185928</v>
+        <v>160994</v>
       </c>
       <c r="H5" s="3">
-        <v>97307</v>
+        <v>96242</v>
       </c>
       <c r="I5" s="4">
-        <v>88621</v>
-      </c>
-      <c r="J5" s="6">
-        <v>33.56</v>
+        <v>64752</v>
+      </c>
+      <c r="J5" s="9">
+        <v>15.396666666666668</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C6" s="3">
-        <v>96641</v>
+        <v>14669</v>
       </c>
       <c r="D6" s="3">
-        <v>15211</v>
-      </c>
-      <c r="E6" s="4">
-        <v>81430</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>20</v>
+        <v>22554</v>
+      </c>
+      <c r="E6" s="7">
+        <v>-7885</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>19</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="6"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3">
-        <v>46296</v>
+        <v>70453</v>
       </c>
       <c r="D7" s="3">
-        <v>44436</v>
+        <v>28994</v>
       </c>
       <c r="E7" s="4">
-        <v>1860</v>
+        <v>41459</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>21</v>
@@ -496,136 +499,136 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="6"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3">
-        <v>85075</v>
+        <v>97745</v>
       </c>
       <c r="D8" s="3">
-        <v>42552</v>
+        <v>10090</v>
       </c>
       <c r="E8" s="4">
-        <v>42523</v>
+        <v>87655</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G8" s="3">
-        <v>199294</v>
+        <v>232186</v>
       </c>
       <c r="H8" s="3">
-        <v>130754</v>
+        <v>86752</v>
       </c>
       <c r="I8" s="4">
-        <v>68540</v>
-      </c>
-      <c r="J8" s="6">
-        <v>22.293333333333333</v>
+        <v>145434</v>
+      </c>
+      <c r="J8" s="9">
+        <v>57.00333333333333</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C9" s="3">
-        <v>32332</v>
+        <v>60378</v>
       </c>
       <c r="D9" s="3">
-        <v>40278</v>
-      </c>
-      <c r="E9" s="7">
-        <v>-7946</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>23</v>
+        <v>49549</v>
+      </c>
+      <c r="E9" s="4">
+        <v>10829</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="6"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3">
-        <v>81887</v>
+        <v>74063</v>
       </c>
       <c r="D10" s="3">
-        <v>47924</v>
+        <v>27113</v>
       </c>
       <c r="E10" s="4">
-        <v>33963</v>
+        <v>46950</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="6"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C11" s="3">
-        <v>39784</v>
+        <v>31660</v>
       </c>
       <c r="D11" s="3">
-        <v>17034</v>
-      </c>
-      <c r="E11" s="4">
-        <v>22750</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>26</v>
+        <v>34289</v>
+      </c>
+      <c r="E11" s="7">
+        <v>-2629</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>28</v>
       </c>
       <c r="G11" s="3">
-        <v>85780</v>
+        <v>139430</v>
       </c>
       <c r="H11" s="3">
-        <v>98157</v>
-      </c>
-      <c r="I11" s="7">
-        <v>-12377</v>
+        <v>97717</v>
+      </c>
+      <c r="I11" s="4">
+        <v>41713</v>
       </c>
       <c r="J11" s="9">
-        <v>-40.919999999999995</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C12" s="3">
-        <v>14944</v>
+        <v>37638</v>
       </c>
       <c r="D12" s="3">
-        <v>34193</v>
-      </c>
-      <c r="E12" s="7">
-        <v>-19249</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>27</v>
+        <v>20848</v>
+      </c>
+      <c r="E12" s="4">
+        <v>16790</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="7"/>
+      <c r="I12" s="4"/>
       <c r="J12" s="9"/>
     </row>
     <row r="13" ht="30" customHeight="1">
@@ -634,204 +637,204 @@
         <v>18</v>
       </c>
       <c r="C13" s="3">
-        <v>31052</v>
+        <v>70132</v>
       </c>
       <c r="D13" s="3">
-        <v>46930</v>
-      </c>
-      <c r="E13" s="7">
-        <v>-15878</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>28</v>
+        <v>42580</v>
+      </c>
+      <c r="E13" s="4">
+        <v>27552</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
-      <c r="I13" s="7"/>
+      <c r="I13" s="4"/>
       <c r="J13" s="9"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C14" s="3">
-        <v>74126</v>
+        <v>82073</v>
       </c>
       <c r="D14" s="3">
-        <v>11871</v>
+        <v>47286</v>
       </c>
       <c r="E14" s="4">
-        <v>62255</v>
+        <v>34787</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G14" s="3">
-        <v>235505</v>
+        <v>224905</v>
       </c>
       <c r="H14" s="3">
-        <v>87212</v>
+        <v>112941</v>
       </c>
       <c r="I14" s="4">
-        <v>148293</v>
-      </c>
-      <c r="J14" s="6">
-        <v>63.166666666666664</v>
+        <v>111964</v>
+      </c>
+      <c r="J14" s="9">
+        <v>49.82333333333333</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C15" s="3">
-        <v>88339</v>
+        <v>65761</v>
       </c>
       <c r="D15" s="3">
-        <v>36497</v>
+        <v>34651</v>
       </c>
       <c r="E15" s="4">
-        <v>51842</v>
+        <v>31110</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="4"/>
-      <c r="J15" s="6"/>
+      <c r="J15" s="9"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>73040</v>
+        <v>77071</v>
       </c>
       <c r="D16" s="3">
-        <v>38844</v>
+        <v>31004</v>
       </c>
       <c r="E16" s="4">
-        <v>34196</v>
+        <v>46067</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="4"/>
-      <c r="J16" s="6"/>
+      <c r="J16" s="9"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C17" s="3">
-        <v>15246</v>
+        <v>38156</v>
       </c>
       <c r="D17" s="3">
-        <v>46641</v>
-      </c>
-      <c r="E17" s="7">
-        <v>-31395</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>34</v>
+        <v>25998</v>
+      </c>
+      <c r="E17" s="4">
+        <v>12158</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="G17" s="3">
-        <v>193758</v>
+        <v>146424</v>
       </c>
       <c r="H17" s="3">
-        <v>103197</v>
+        <v>90773</v>
       </c>
       <c r="I17" s="4">
-        <v>90561</v>
-      </c>
-      <c r="J17" s="9">
-        <v>-23.239999999999995</v>
+        <v>55651</v>
+      </c>
+      <c r="J17" s="6">
+        <v>-43.48333333333334</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C18" s="3">
-        <v>82309</v>
+        <v>12065</v>
       </c>
       <c r="D18" s="3">
-        <v>28549</v>
-      </c>
-      <c r="E18" s="4">
-        <v>53760</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>35</v>
+        <v>40693</v>
+      </c>
+      <c r="E18" s="7">
+        <v>-28628</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>36</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="4"/>
-      <c r="J18" s="9"/>
+      <c r="J18" s="6"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C19" s="3">
         <v>96203</v>
       </c>
       <c r="D19" s="3">
-        <v>28007</v>
+        <v>24082</v>
       </c>
       <c r="E19" s="4">
-        <v>68196</v>
+        <v>72121</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="9"/>
+      <c r="J19" s="6"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C20" s="3">
-        <v>95353</v>
+        <v>40115</v>
       </c>
       <c r="D20" s="3">
-        <v>18276</v>
+        <v>39020</v>
       </c>
       <c r="E20" s="4">
-        <v>77077</v>
+        <v>1095</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G20" s="3">
-        <v>171035</v>
+        <v>127355</v>
       </c>
       <c r="H20" s="3">
-        <v>64401</v>
+        <v>116827</v>
       </c>
       <c r="I20" s="4">
-        <v>106634</v>
+        <v>10528</v>
       </c>
       <c r="J20" s="6">
-        <v>54.23333333333333</v>
+        <v>-16.009999999999998</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -840,16 +843,16 @@
         <v>24</v>
       </c>
       <c r="C21" s="3">
-        <v>20824</v>
+        <v>21315</v>
       </c>
       <c r="D21" s="3">
-        <v>11428</v>
-      </c>
-      <c r="E21" s="4">
-        <v>9396</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>39</v>
+        <v>41812</v>
+      </c>
+      <c r="E21" s="7">
+        <v>-20497</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
@@ -859,19 +862,19 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C22" s="3">
-        <v>54858</v>
+        <v>65925</v>
       </c>
       <c r="D22" s="3">
-        <v>34697</v>
+        <v>35995</v>
       </c>
       <c r="E22" s="4">
-        <v>20161</v>
+        <v>29930</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
@@ -880,133 +883,133 @@
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C23" s="3">
-        <v>67786</v>
+        <v>62823</v>
       </c>
       <c r="D23" s="3">
-        <v>37730</v>
+        <v>11395</v>
       </c>
       <c r="E23" s="4">
-        <v>30056</v>
+        <v>51428</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G23" s="3">
-        <v>216938</v>
+        <v>168546</v>
       </c>
       <c r="H23" s="3">
-        <v>73385</v>
+        <v>87116</v>
       </c>
       <c r="I23" s="4">
-        <v>143553</v>
-      </c>
-      <c r="J23" s="6">
-        <v>64.51333333333334</v>
+        <v>81430</v>
+      </c>
+      <c r="J23" s="9">
+        <v>33.080000000000005</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C24" s="3">
-        <v>68128</v>
+        <v>79464</v>
       </c>
       <c r="D24" s="3">
-        <v>29100</v>
+        <v>41472</v>
       </c>
       <c r="E24" s="4">
-        <v>39028</v>
+        <v>37992</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="6"/>
+      <c r="J24" s="9"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C25" s="3">
-        <v>81024</v>
+        <v>26259</v>
       </c>
       <c r="D25" s="3">
-        <v>6555</v>
-      </c>
-      <c r="E25" s="4">
-        <v>74469</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>43</v>
+        <v>34249</v>
+      </c>
+      <c r="E25" s="7">
+        <v>-7990</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="6"/>
+      <c r="J25" s="9"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C26" s="3">
-        <v>65895</v>
+        <v>12409</v>
       </c>
       <c r="D26" s="3">
-        <v>9058</v>
-      </c>
-      <c r="E26" s="4">
-        <v>56837</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>45</v>
+        <v>29553</v>
+      </c>
+      <c r="E26" s="7">
+        <v>-17144</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>46</v>
       </c>
       <c r="G26" s="3">
-        <v>204870</v>
+        <v>155008</v>
       </c>
       <c r="H26" s="3">
-        <v>29398</v>
+        <v>53294</v>
       </c>
       <c r="I26" s="4">
-        <v>175472</v>
-      </c>
-      <c r="J26" s="6">
-        <v>85.33999999999999</v>
+        <v>101714</v>
+      </c>
+      <c r="J26" s="9">
+        <v>9.453333333333338</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C27" s="3">
-        <v>74370</v>
+        <v>76909</v>
       </c>
       <c r="D27" s="3">
-        <v>6131</v>
+        <v>11994</v>
       </c>
       <c r="E27" s="4">
-        <v>68239</v>
+        <v>64915</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="4"/>
-      <c r="J27" s="6"/>
+      <c r="J27" s="9"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2"/>
@@ -1014,52 +1017,52 @@
         <v>24</v>
       </c>
       <c r="C28" s="3">
-        <v>64605</v>
+        <v>65690</v>
       </c>
       <c r="D28" s="3">
-        <v>14209</v>
+        <v>11747</v>
       </c>
       <c r="E28" s="4">
-        <v>50396</v>
+        <v>53943</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="4"/>
-      <c r="J28" s="6"/>
+      <c r="J28" s="9"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C29" s="3">
-        <v>13464</v>
+        <v>80374</v>
       </c>
       <c r="D29" s="3">
-        <v>27598</v>
-      </c>
-      <c r="E29" s="7">
-        <v>-14134</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>48</v>
+        <v>37375</v>
+      </c>
+      <c r="E29" s="4">
+        <v>42999</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="G29" s="3">
-        <v>124441</v>
+        <v>150985</v>
       </c>
       <c r="H29" s="3">
-        <v>72076</v>
+        <v>91542</v>
       </c>
       <c r="I29" s="4">
-        <v>52365</v>
+        <v>59443</v>
       </c>
       <c r="J29" s="9">
-        <v>-4.026666666666666</v>
+        <v>19.573333333333334</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
@@ -1068,16 +1071,16 @@
         <v>11</v>
       </c>
       <c r="C30" s="3">
-        <v>72158</v>
+        <v>14158</v>
       </c>
       <c r="D30" s="3">
-        <v>6284</v>
-      </c>
-      <c r="E30" s="4">
-        <v>65874</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>49</v>
+        <v>18676</v>
+      </c>
+      <c r="E30" s="7">
+        <v>-4518</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>50</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -1087,19 +1090,19 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C31" s="3">
-        <v>38819</v>
+        <v>56453</v>
       </c>
       <c r="D31" s="3">
-        <v>38194</v>
+        <v>35491</v>
       </c>
       <c r="E31" s="4">
-        <v>625</v>
+        <v>20962</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
@@ -1108,16 +1111,16 @@
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1719034</v>
+        <v>1604190</v>
       </c>
       <c r="H32" s="10">
-        <v>794791</v>
+        <v>915636</v>
       </c>
       <c r="I32" s="11">
-        <v>924243</v>
+        <v>688554</v>
       </c>
       <c r="J32" s="12">
-        <v>30.624333333333333</v>
+        <v>13.806333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(core): checkpoint excel table grouped formulas
</commit_message>
<xml_diff>
--- a/packages/typed-xlsx/examples/financial-report.xlsx
+++ b/packages/typed-xlsx/examples/financial-report.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>Month</t>
   </si>
@@ -40,130 +40,127 @@
     <t>Average Profit Margin</t>
   </si>
   <si>
+    <t>2023-08</t>
+  </si>
+  <si>
+    <t>R&amp;D</t>
+  </si>
+  <si>
+    <t>53.27%</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>67.8%</t>
+  </si>
+  <si>
+    <t>78.17%</t>
+  </si>
+  <si>
+    <t>2023-09</t>
+  </si>
+  <si>
+    <t>Customer Support</t>
+  </si>
+  <si>
+    <t>78.06%</t>
+  </si>
+  <si>
+    <t>85.95%</t>
+  </si>
+  <si>
+    <t>50.51%</t>
+  </si>
+  <si>
+    <t>2023-10</t>
+  </si>
+  <si>
+    <t>90.08%</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>85.2%</t>
+  </si>
+  <si>
+    <t>81%</t>
+  </si>
+  <si>
+    <t>56.46%</t>
+  </si>
+  <si>
+    <t>29.26%</t>
+  </si>
+  <si>
+    <t>93.74%</t>
+  </si>
+  <si>
+    <t>41.15%</t>
+  </si>
+  <si>
+    <t>79.25%</t>
+  </si>
+  <si>
+    <t>-127.02%</t>
+  </si>
+  <si>
+    <t>87.65%</t>
+  </si>
+  <si>
+    <t>36.79%</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>87.17%</t>
+  </si>
+  <si>
     <t>2023-11</t>
   </si>
   <si>
-    <t>Human Resources</t>
-  </si>
-  <si>
-    <t>9.86%</t>
-  </si>
-  <si>
-    <t>Marketing</t>
-  </si>
-  <si>
-    <t>52.77%</t>
-  </si>
-  <si>
-    <t>-98.55%</t>
+    <t>9.43%</t>
+  </si>
+  <si>
+    <t>25.21%</t>
+  </si>
+  <si>
+    <t>54.75%</t>
+  </si>
+  <si>
+    <t>2023-03</t>
+  </si>
+  <si>
+    <t>68.2%</t>
+  </si>
+  <si>
+    <t>65.83%</t>
+  </si>
+  <si>
+    <t>52.63%</t>
   </si>
   <si>
     <t>2023-12</t>
   </si>
   <si>
-    <t>41.09%</t>
-  </si>
-  <si>
-    <t>R&amp;D</t>
-  </si>
-  <si>
-    <t>-53.75%</t>
-  </si>
-  <si>
-    <t>Customer Support</t>
-  </si>
-  <si>
-    <t>58.85%</t>
-  </si>
-  <si>
-    <t>2023-05</t>
-  </si>
-  <si>
-    <t>89.68%</t>
-  </si>
-  <si>
-    <t>Sales</t>
-  </si>
-  <si>
-    <t>17.94%</t>
-  </si>
-  <si>
-    <t>63.39%</t>
-  </si>
-  <si>
-    <t>2023-08</t>
-  </si>
-  <si>
-    <t>-8.3%</t>
-  </si>
-  <si>
-    <t>44.61%</t>
-  </si>
-  <si>
-    <t>39.29%</t>
-  </si>
-  <si>
-    <t>42.39%</t>
-  </si>
-  <si>
-    <t>47.31%</t>
-  </si>
-  <si>
-    <t>59.77%</t>
-  </si>
-  <si>
-    <t>2023-10</t>
-  </si>
-  <si>
-    <t>31.86%</t>
-  </si>
-  <si>
-    <t>-237.28%</t>
-  </si>
-  <si>
-    <t>74.97%</t>
-  </si>
-  <si>
-    <t>2023-04</t>
-  </si>
-  <si>
-    <t>2.73%</t>
-  </si>
-  <si>
-    <t>-96.16%</t>
-  </si>
-  <si>
-    <t>45.4%</t>
-  </si>
-  <si>
-    <t>81.86%</t>
-  </si>
-  <si>
-    <t>47.81%</t>
-  </si>
-  <si>
-    <t>-30.43%</t>
-  </si>
-  <si>
-    <t>2023-09</t>
-  </si>
-  <si>
-    <t>-138.16%</t>
-  </si>
-  <si>
-    <t>84.4%</t>
-  </si>
-  <si>
-    <t>82.12%</t>
-  </si>
-  <si>
-    <t>53.5%</t>
-  </si>
-  <si>
-    <t>-31.91%</t>
-  </si>
-  <si>
-    <t>37.13%</t>
+    <t>58.55%</t>
+  </si>
+  <si>
+    <t>-40.05%</t>
+  </si>
+  <si>
+    <t>45.63%</t>
+  </si>
+  <si>
+    <t>65.3%</t>
+  </si>
+  <si>
+    <t>77.01%</t>
+  </si>
+  <si>
+    <t>93.1%</t>
   </si>
 </sst>
 </file>
@@ -272,6 +269,9 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -279,9 +279,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -357,28 +354,28 @@
         <v>11</v>
       </c>
       <c r="C2" s="3">
-        <v>37960</v>
+        <v>54380</v>
       </c>
       <c r="D2" s="3">
-        <v>34219</v>
+        <v>25414</v>
       </c>
       <c r="E2" s="4">
-        <v>3741</v>
+        <v>28966</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>12</v>
       </c>
       <c r="G2" s="3">
-        <v>98357</v>
+        <v>167977</v>
       </c>
       <c r="H2" s="3">
-        <v>82432</v>
+        <v>55764</v>
       </c>
       <c r="I2" s="4">
-        <v>15925</v>
+        <v>112213</v>
       </c>
       <c r="J2" s="6">
-        <v>-11.973333333333331</v>
+        <v>66.41333333333334</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -387,13 +384,13 @@
         <v>13</v>
       </c>
       <c r="C3" s="3">
-        <v>47388</v>
+        <v>53509</v>
       </c>
       <c r="D3" s="3">
-        <v>22383</v>
+        <v>17231</v>
       </c>
       <c r="E3" s="4">
-        <v>25005</v>
+        <v>36278</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>14</v>
@@ -409,15 +406,15 @@
         <v>11</v>
       </c>
       <c r="C4" s="3">
-        <v>13009</v>
+        <v>60088</v>
       </c>
       <c r="D4" s="3">
-        <v>25830</v>
-      </c>
-      <c r="E4" s="7">
-        <v>-12821</v>
-      </c>
-      <c r="F4" s="8" t="s">
+        <v>13119</v>
+      </c>
+      <c r="E4" s="4">
+        <v>46969</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G4" s="3"/>
@@ -430,335 +427,335 @@
         <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C5" s="3">
-        <v>75872</v>
+        <v>79673</v>
       </c>
       <c r="D5" s="3">
-        <v>44694</v>
+        <v>17478</v>
       </c>
       <c r="E5" s="4">
-        <v>31178</v>
+        <v>62195</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G5" s="3">
-        <v>160994</v>
+        <v>214543</v>
       </c>
       <c r="H5" s="3">
-        <v>96242</v>
+        <v>50219</v>
       </c>
       <c r="I5" s="4">
-        <v>64752</v>
-      </c>
-      <c r="J5" s="9">
-        <v>15.396666666666668</v>
+        <v>164324</v>
+      </c>
+      <c r="J5" s="6">
+        <v>71.50666666666666</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C6" s="3">
-        <v>14669</v>
+        <v>95948</v>
       </c>
       <c r="D6" s="3">
-        <v>22554</v>
-      </c>
-      <c r="E6" s="7">
-        <v>-7885</v>
-      </c>
-      <c r="F6" s="8" t="s">
+        <v>13480</v>
+      </c>
+      <c r="E6" s="4">
+        <v>82468</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="4"/>
-      <c r="J6" s="9"/>
+      <c r="J6" s="6"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3">
+        <v>38922</v>
+      </c>
+      <c r="D7" s="3">
+        <v>19261</v>
+      </c>
+      <c r="E7" s="4">
+        <v>19661</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="C7" s="3">
-        <v>70453</v>
-      </c>
-      <c r="D7" s="3">
-        <v>28994</v>
-      </c>
-      <c r="E7" s="4">
-        <v>41459</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>21</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="9"/>
+      <c r="J7" s="6"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="3">
-        <v>97745</v>
+        <v>74870</v>
       </c>
       <c r="D8" s="3">
-        <v>10090</v>
+        <v>7430</v>
       </c>
       <c r="E8" s="4">
-        <v>87655</v>
+        <v>67440</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G8" s="3">
-        <v>232186</v>
+        <v>242036</v>
       </c>
       <c r="H8" s="3">
-        <v>86752</v>
+        <v>35525</v>
       </c>
       <c r="I8" s="4">
-        <v>145434</v>
-      </c>
-      <c r="J8" s="9">
-        <v>57.00333333333333</v>
+        <v>206511</v>
+      </c>
+      <c r="J8" s="6">
+        <v>85.42666666666666</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="3">
+        <v>87264</v>
+      </c>
+      <c r="D9" s="3">
+        <v>12914</v>
+      </c>
+      <c r="E9" s="4">
+        <v>74350</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="C9" s="3">
-        <v>60378</v>
-      </c>
-      <c r="D9" s="3">
-        <v>49549</v>
-      </c>
-      <c r="E9" s="4">
-        <v>10829</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
-      <c r="J9" s="9"/>
+      <c r="J9" s="6"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="C10" s="3">
-        <v>74063</v>
+        <v>79902</v>
       </c>
       <c r="D10" s="3">
-        <v>27113</v>
+        <v>15181</v>
       </c>
       <c r="E10" s="4">
-        <v>46950</v>
+        <v>64721</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
-      <c r="J10" s="9"/>
+      <c r="J10" s="6"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C11" s="3">
-        <v>31660</v>
+        <v>51827</v>
       </c>
       <c r="D11" s="3">
-        <v>34289</v>
-      </c>
-      <c r="E11" s="7">
-        <v>-2629</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>28</v>
+        <v>22566</v>
+      </c>
+      <c r="E11" s="4">
+        <v>29261</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="G11" s="3">
-        <v>139430</v>
+        <v>190297</v>
       </c>
       <c r="H11" s="3">
-        <v>97717</v>
+        <v>65155</v>
       </c>
       <c r="I11" s="4">
-        <v>41713</v>
-      </c>
-      <c r="J11" s="9">
-        <v>25.2</v>
+        <v>125142</v>
+      </c>
+      <c r="J11" s="6">
+        <v>59.81999999999999</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C12" s="3">
-        <v>37638</v>
+        <v>52615</v>
       </c>
       <c r="D12" s="3">
-        <v>20848</v>
+        <v>37218</v>
       </c>
       <c r="E12" s="4">
-        <v>16790</v>
+        <v>15397</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="9"/>
+      <c r="J12" s="6"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C13" s="3">
-        <v>70132</v>
+        <v>85855</v>
       </c>
       <c r="D13" s="3">
-        <v>42580</v>
+        <v>5371</v>
       </c>
       <c r="E13" s="4">
-        <v>27552</v>
+        <v>80484</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="9"/>
+      <c r="J13" s="6"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C14" s="3">
-        <v>82073</v>
+        <v>28818</v>
       </c>
       <c r="D14" s="3">
-        <v>47286</v>
+        <v>16958</v>
       </c>
       <c r="E14" s="4">
-        <v>34787</v>
+        <v>11860</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G14" s="3">
-        <v>224905</v>
+        <v>126065</v>
       </c>
       <c r="H14" s="3">
-        <v>112941</v>
+        <v>72493</v>
       </c>
       <c r="I14" s="4">
-        <v>111964</v>
-      </c>
-      <c r="J14" s="9">
-        <v>49.82333333333333</v>
+        <v>53572</v>
+      </c>
+      <c r="J14" s="7">
+        <v>-2.2066666666666634</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C15" s="3">
-        <v>65761</v>
+        <v>80108</v>
       </c>
       <c r="D15" s="3">
-        <v>34651</v>
+        <v>16626</v>
       </c>
       <c r="E15" s="4">
-        <v>31110</v>
+        <v>63482</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="4"/>
-      <c r="J15" s="9"/>
+      <c r="J15" s="7"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C16" s="3">
-        <v>77071</v>
+        <v>17139</v>
       </c>
       <c r="D16" s="3">
-        <v>31004</v>
-      </c>
-      <c r="E16" s="4">
-        <v>46067</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>33</v>
+        <v>38909</v>
+      </c>
+      <c r="E16" s="8">
+        <v>-21770</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>31</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="4"/>
-      <c r="J16" s="9"/>
+      <c r="J16" s="7"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C17" s="3">
-        <v>38156</v>
+        <v>84430</v>
       </c>
       <c r="D17" s="3">
-        <v>25998</v>
+        <v>10424</v>
       </c>
       <c r="E17" s="4">
-        <v>12158</v>
+        <v>74006</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G17" s="3">
-        <v>146424</v>
+        <v>239004</v>
       </c>
       <c r="H17" s="3">
-        <v>90773</v>
+        <v>64137</v>
       </c>
       <c r="I17" s="4">
-        <v>55651</v>
+        <v>174867</v>
       </c>
       <c r="J17" s="6">
-        <v>-43.48333333333334</v>
+        <v>70.53666666666668</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
@@ -767,16 +764,16 @@
         <v>11</v>
       </c>
       <c r="C18" s="3">
-        <v>12065</v>
+        <v>67244</v>
       </c>
       <c r="D18" s="3">
-        <v>40693</v>
-      </c>
-      <c r="E18" s="7">
-        <v>-28628</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>36</v>
+        <v>42508</v>
+      </c>
+      <c r="E18" s="4">
+        <v>24736</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>33</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
@@ -786,19 +783,19 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="2"/>
       <c r="B19" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C19" s="3">
-        <v>96203</v>
+        <v>87330</v>
       </c>
       <c r="D19" s="3">
-        <v>24082</v>
+        <v>11205</v>
       </c>
       <c r="E19" s="4">
-        <v>72121</v>
+        <v>76125</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
@@ -807,52 +804,52 @@
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C20" s="3">
-        <v>40115</v>
+        <v>13148</v>
       </c>
       <c r="D20" s="3">
-        <v>39020</v>
+        <v>11908</v>
       </c>
       <c r="E20" s="4">
-        <v>1095</v>
+        <v>1240</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G20" s="3">
-        <v>127355</v>
+        <v>117880</v>
       </c>
       <c r="H20" s="3">
-        <v>116827</v>
+        <v>67662</v>
       </c>
       <c r="I20" s="4">
-        <v>10528</v>
+        <v>50218</v>
       </c>
       <c r="J20" s="6">
-        <v>-16.009999999999998</v>
+        <v>29.796666666666667</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C21" s="3">
-        <v>21315</v>
+        <v>28307</v>
       </c>
       <c r="D21" s="3">
-        <v>41812</v>
-      </c>
-      <c r="E21" s="7">
-        <v>-20497</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>40</v>
+        <v>21170</v>
+      </c>
+      <c r="E21" s="4">
+        <v>7137</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
@@ -865,16 +862,16 @@
         <v>11</v>
       </c>
       <c r="C22" s="3">
-        <v>65925</v>
+        <v>76425</v>
       </c>
       <c r="D22" s="3">
-        <v>35995</v>
+        <v>34584</v>
       </c>
       <c r="E22" s="4">
-        <v>29930</v>
+        <v>41841</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
@@ -883,209 +880,209 @@
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="C23" s="3">
-        <v>62823</v>
+        <v>45867</v>
       </c>
       <c r="D23" s="3">
-        <v>11395</v>
+        <v>14584</v>
       </c>
       <c r="E23" s="4">
-        <v>51428</v>
+        <v>31283</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G23" s="3">
-        <v>168546</v>
+        <v>211658</v>
       </c>
       <c r="H23" s="3">
-        <v>87116</v>
+        <v>82695</v>
       </c>
       <c r="I23" s="4">
-        <v>81430</v>
-      </c>
-      <c r="J23" s="9">
-        <v>33.080000000000005</v>
+        <v>128963</v>
+      </c>
+      <c r="J23" s="6">
+        <v>62.22</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C24" s="3">
-        <v>79464</v>
+        <v>78962</v>
       </c>
       <c r="D24" s="3">
-        <v>41472</v>
+        <v>26983</v>
       </c>
       <c r="E24" s="4">
-        <v>37992</v>
+        <v>51979</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="9"/>
+      <c r="J24" s="6"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C25" s="3">
-        <v>26259</v>
+        <v>86829</v>
       </c>
       <c r="D25" s="3">
-        <v>34249</v>
-      </c>
-      <c r="E25" s="7">
-        <v>-7990</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>44</v>
+        <v>41128</v>
+      </c>
+      <c r="E25" s="4">
+        <v>45701</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="9"/>
+      <c r="J25" s="6"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="3">
+        <v>66249</v>
+      </c>
+      <c r="D26" s="3">
+        <v>27462</v>
+      </c>
+      <c r="E26" s="4">
+        <v>38787</v>
+      </c>
+      <c r="F26" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" s="3">
-        <v>12409</v>
-      </c>
-      <c r="D26" s="3">
-        <v>29553</v>
-      </c>
-      <c r="E26" s="7">
-        <v>-17144</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>46</v>
-      </c>
       <c r="G26" s="3">
-        <v>155008</v>
+        <v>172042</v>
       </c>
       <c r="H26" s="3">
-        <v>53294</v>
+        <v>100816</v>
       </c>
       <c r="I26" s="4">
-        <v>101714</v>
-      </c>
-      <c r="J26" s="9">
-        <v>9.453333333333338</v>
+        <v>71226</v>
+      </c>
+      <c r="J26" s="6">
+        <v>21.376666666666665</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C27" s="3">
-        <v>76909</v>
+        <v>18480</v>
       </c>
       <c r="D27" s="3">
-        <v>11994</v>
-      </c>
-      <c r="E27" s="4">
-        <v>64915</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>47</v>
+        <v>25881</v>
+      </c>
+      <c r="E27" s="8">
+        <v>-7401</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>46</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="4"/>
-      <c r="J27" s="9"/>
+      <c r="J27" s="6"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C28" s="3">
-        <v>65690</v>
+        <v>87313</v>
       </c>
       <c r="D28" s="3">
-        <v>11747</v>
+        <v>47473</v>
       </c>
       <c r="E28" s="4">
-        <v>53943</v>
+        <v>39840</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="4"/>
-      <c r="J28" s="9"/>
+      <c r="J28" s="6"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C29" s="3">
-        <v>80374</v>
+        <v>98783</v>
       </c>
       <c r="D29" s="3">
-        <v>37375</v>
+        <v>34276</v>
       </c>
       <c r="E29" s="4">
-        <v>42999</v>
+        <v>64507</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G29" s="3">
-        <v>150985</v>
+        <v>252261</v>
       </c>
       <c r="H29" s="3">
-        <v>91542</v>
+        <v>56015</v>
       </c>
       <c r="I29" s="4">
-        <v>59443</v>
-      </c>
-      <c r="J29" s="9">
-        <v>19.573333333333334</v>
+        <v>196246</v>
+      </c>
+      <c r="J29" s="6">
+        <v>78.47</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="C30" s="3">
-        <v>14158</v>
+        <v>69291</v>
       </c>
       <c r="D30" s="3">
-        <v>18676</v>
-      </c>
-      <c r="E30" s="7">
-        <v>-4518</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>50</v>
+        <v>15932</v>
+      </c>
+      <c r="E30" s="4">
+        <v>53359</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="4"/>
-      <c r="J30" s="9"/>
+      <c r="J30" s="6"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="2"/>
@@ -1093,34 +1090,34 @@
         <v>13</v>
       </c>
       <c r="C31" s="3">
-        <v>56453</v>
+        <v>84187</v>
       </c>
       <c r="D31" s="3">
-        <v>35491</v>
+        <v>5807</v>
       </c>
       <c r="E31" s="4">
-        <v>20962</v>
+        <v>78380</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="4"/>
-      <c r="J31" s="9"/>
+      <c r="J31" s="6"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="G32" s="10">
-        <v>1604190</v>
+        <v>1933763</v>
       </c>
       <c r="H32" s="10">
-        <v>915636</v>
+        <v>650481</v>
       </c>
       <c r="I32" s="11">
-        <v>688554</v>
+        <v>1283282</v>
       </c>
       <c r="J32" s="12">
-        <v>13.806333333333333</v>
+        <v>54.33600000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>